<commit_message>
Update initial populations and estimates
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPathsFork\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F019F217-8606-4580-9514-E6F1BFECDEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFC10CB-0383-400D-AE66-8078D9FB660D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="17363" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -182,10 +182,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,14 +469,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.73046875" customWidth="1"/>
+    <col min="2" max="2" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -484,50 +484,50 @@
         <v>44593</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -540,12 +540,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530F7AD6-02C1-41F5-9B11-F88D7B76E795}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -553,7 +553,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -561,7 +561,7 @@
         <v>0.5511963385465366</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -569,7 +569,7 @@
         <v>0.56378226458419012</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -577,7 +577,7 @@
         <v>0.3588496779494994</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -585,7 +585,7 @@
         <v>0.37499140584966989</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -593,7 +593,7 @@
         <v>2.4158001968775116</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -601,7 +601,7 @@
         <v>1.8361431734912119</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -609,7 +609,7 @@
         <v>1.5969934128957666</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -617,7 +617,7 @@
         <v>884.81552442493353</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -625,7 +625,7 @@
         <v>1.528311</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -633,7 +633,7 @@
         <v>1.1671</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -641,7 +641,7 @@
         <v>1.2093</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -649,7 +649,7 @@
         <v>0.98887999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -657,7 +657,7 @@
         <v>0.95128999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -665,7 +665,7 @@
         <v>0.84714999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -673,7 +673,7 @@
         <v>0.94330000000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -681,7 +681,7 @@
         <v>1.2788999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -697,9 +697,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA17ED43-A333-4863-9108-47B84B48F4F1}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -707,7 +707,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -715,7 +715,7 @@
         <v>0.53371000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -723,7 +723,7 @@
         <v>0.64690999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -731,7 +731,7 @@
         <v>5.4573999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -739,7 +739,7 @@
         <v>3.2025999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -747,7 +747,7 @@
         <v>2.4695999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -755,7 +755,7 @@
         <v>1.5126999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -763,7 +763,7 @@
         <v>1.4134</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -771,7 +771,7 @@
         <v>1.1671</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -779,7 +779,7 @@
         <v>0.58166506869277523</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -795,66 +795,66 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B52D91-862E-459C-B8A1-E5C1A5D5C4F0}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="5" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="20.265625" style="4" customWidth="1"/>
+    <col min="2" max="16384" width="9.1328125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="5">
-        <v>0.93612804771750313</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="B2">
+        <v>0.62469531038656967</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="5">
-        <v>0.94686376540135364</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="B3">
+        <v>0.77537096517828041</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="5">
-        <v>0.41369964379833796</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="B4">
+        <v>0.42903109977918413</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
-        <v>0.46915379886598663</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B5">
+        <v>0.51863601752897992</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5">
-        <v>1.0047416470996766</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="B6">
+        <v>1.1567001834965824</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="5">
-        <v>1.0352761099546386</v>
+      <c r="B7">
+        <v>1.1849409507270041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RMSE and union matching parameters
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E294D63C-8817-4073-A78B-9A51773CAA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B203BA80-3954-48F2-876D-7720C5B35E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
     <sheet name="UK" sheetId="2" r:id="rId2"/>
     <sheet name="IT" sheetId="3" r:id="rId3"/>
     <sheet name="PL" sheetId="4" r:id="rId4"/>
+    <sheet name="EL" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="22">
   <si>
     <t>Date modified</t>
   </si>
@@ -448,14 +449,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" customWidth="1"/>
-    <col min="2" max="2" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.3984375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -463,7 +464,7 @@
         <v>44593</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -476,7 +477,7 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -484,7 +485,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -492,7 +493,7 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -500,7 +501,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -519,12 +520,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530F7AD6-02C1-41F5-9B11-F88D7B76E795}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -532,7 +533,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -540,7 +541,7 @@
         <v>0.5511963385465366</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -548,7 +549,7 @@
         <v>0.56378226458419012</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -556,7 +557,7 @@
         <v>0.3588496779494994</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -564,7 +565,7 @@
         <v>0.37499140584966989</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -572,7 +573,7 @@
         <v>2.4158001968775116</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -580,7 +581,7 @@
         <v>1.8361431734912119</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -588,7 +589,7 @@
         <v>1.5969934128957666</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -596,7 +597,7 @@
         <v>884.81552442493353</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -604,7 +605,7 @@
         <v>1.528311</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -612,7 +613,7 @@
         <v>1.1671</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -620,7 +621,7 @@
         <v>1.2093</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -628,7 +629,7 @@
         <v>0.98887999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -636,7 +637,7 @@
         <v>0.95128999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -644,7 +645,7 @@
         <v>0.84714999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -652,7 +653,7 @@
         <v>0.94330000000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -660,7 +661,7 @@
         <v>1.2788999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -676,12 +677,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA17ED43-A333-4863-9108-47B84B48F4F1}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -689,7 +690,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -697,7 +698,7 @@
         <v>0.78402799000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -705,7 +706,7 @@
         <v>0.780405829</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -713,7 +714,7 @@
         <v>0.41129760100000001</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -721,7 +722,7 @@
         <v>0.42725606100000002</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -729,7 +730,7 @@
         <v>1.656046431</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -737,10 +738,10 @@
         <v>1.389078416</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="3"/>
     </row>
   </sheetData>
@@ -751,13 +752,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B52D91-862E-459C-B8A1-E5C1A5D5C4F0}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.265625" style="4" customWidth="1"/>
-    <col min="2" max="16384" width="9.1328125" style="4"/>
+    <col min="1" max="1" width="20.28515625" style="4" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -765,7 +766,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
@@ -773,7 +774,7 @@
         <v>0.77710092075167148</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -781,7 +782,7 @@
         <v>0.80966819962611325</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
@@ -789,7 +790,7 @@
         <v>0.40685676867032922</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -797,7 +798,7 @@
         <v>0.48603505601304164</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -805,12 +806,78 @@
         <v>1.0366294171387864</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B7">
         <v>1.0108885888661292</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893BB49F-CF19-4603-AFB7-6E78A149B7C0}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>0.68700237315658907</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>0.60980188127721924</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>0.44340598457435321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>0.41540500765020927</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1.656046431</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1.389078416</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new regression files #154
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/Documents/GitHub/SimPathsFork/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8D1E43-29B4-4F4F-A480-671D21A6423A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0B37DB-0F66-4AC3-A395-98E72F05568E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5500" yWindow="1760" windowWidth="17420" windowHeight="17220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -76,7 +76,49 @@
     <t>S3e</t>
   </si>
   <si>
-    <t>HM1</t>
+    <t>HM1_L</t>
+  </si>
+  <si>
+    <t>HM2_Females_L</t>
+  </si>
+  <si>
+    <t>HM2_Males_L</t>
+  </si>
+  <si>
+    <t>HM1_C</t>
+  </si>
+  <si>
+    <t>HM2_Females_C</t>
+  </si>
+  <si>
+    <t>HM2_Males_C</t>
+  </si>
+  <si>
+    <t>DHE_MCS1</t>
+  </si>
+  <si>
+    <t>DHE_MCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_MCS2_Males</t>
+  </si>
+  <si>
+    <t>DHE_PCS1</t>
+  </si>
+  <si>
+    <t>DHE_PCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_PCS2_Males</t>
+  </si>
+  <si>
+    <t>DLS1</t>
+  </si>
+  <si>
+    <t>DLS2_Females</t>
+  </si>
+  <si>
+    <t>DLS2_Males</t>
   </si>
 </sst>
 </file>
@@ -451,13 +493,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -465,7 +507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -473,7 +515,7 @@
         <v>0.66454278033706471</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -481,7 +523,7 @@
         <v>0.60703408649523138</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -489,7 +531,7 @@
         <v>0.36022674874857058</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -497,7 +539,7 @@
         <v>0.36081327540689057</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -505,7 +547,7 @@
         <v>2.0896398243248244</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -513,7 +555,7 @@
         <v>1.8775380284661962</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -521,7 +563,7 @@
         <v>0.88807293643925145</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -529,7 +571,7 @@
         <v>1.0339139410534337</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -537,7 +579,7 @@
         <v>1.528311</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -545,7 +587,7 @@
         <v>1.1671</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -553,7 +595,7 @@
         <v>1.2093</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -561,7 +603,7 @@
         <v>0.98887999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -569,7 +611,7 @@
         <v>0.95128999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -577,7 +619,7 @@
         <v>0.84714999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -585,7 +627,7 @@
         <v>0.94330000000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -593,12 +635,124 @@
         <v>1.2788999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="1">
-        <v>4.4850000000000003</v>
+        <v>4.4450300852579687</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1">
+        <v>4.2643450657440756</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1">
+        <v>3.7017614114976105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2.5612048553045885</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2.5438883298479338</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1">
+        <v>2.1461867603136353</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="1">
+        <v>7.951543214267657</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="1">
+        <v>7.2255004634210964</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1">
+        <v>6.4645902205901891</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>7.1364100298230317</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>6.1641660235755289</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>5.4985584120343427</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>1.2179012672192562</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>1.0828588494430789</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>1.0201905534361162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrate new simplified social care module
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27180CD6-FE9B-9445-88F9-015D1CE08367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9555AB-8AA4-D249-978F-9FC3774B729B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -52,24 +52,6 @@
     <t>S1b</t>
   </si>
   <si>
-    <t>S2g</t>
-  </si>
-  <si>
-    <t>S2h</t>
-  </si>
-  <si>
-    <t>S2i</t>
-  </si>
-  <si>
-    <t>S2j</t>
-  </si>
-  <si>
-    <t>S2k</t>
-  </si>
-  <si>
-    <t>S3e</t>
-  </si>
-  <si>
     <t>HM1_L</t>
   </si>
   <si>
@@ -83,6 +65,21 @@
   </si>
   <si>
     <t>C1b</t>
+  </si>
+  <si>
+    <t>S3c</t>
+  </si>
+  <si>
+    <t>S3d</t>
+  </si>
+  <si>
+    <t>S2c</t>
+  </si>
+  <si>
+    <t>S2d</t>
+  </si>
+  <si>
+    <t>S2e</t>
   </si>
 </sst>
 </file>
@@ -457,8 +454,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -534,7 +534,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1">
         <v>1.2093</v>
@@ -542,7 +542,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B11" s="1">
         <v>0.98887999999999998</v>
@@ -550,7 +550,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1">
         <v>0.95128999999999997</v>
@@ -558,65 +558,57 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B13" s="1">
-        <v>0.84714999999999996</v>
+        <v>1.2788999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1">
-        <v>0.94330000000000003</v>
+        <v>1.2788999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B15" s="1">
-        <v>1.2788999999999999</v>
+        <v>4.4450300852579687</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B16" s="1">
-        <v>4.4450300852579687</v>
+        <v>7.951543214267657</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="1">
-        <v>7.951543214267657</v>
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>7.1364100298230317</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B18">
-        <v>7.1364100298230317</v>
+        <v>1.2179012672192562</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19">
-        <v>1.2179012672192562</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="1">
+      <c r="A19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="1">
         <v>1.528311</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update financial distress and health process estimates
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eii2t\src\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9555AB-8AA4-D249-978F-9FC3774B729B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97D79955-02FD-4CC6-8C7B-2EC59B60F1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -80,6 +80,39 @@
   </si>
   <si>
     <t>S2e</t>
+  </si>
+  <si>
+    <t>HM2_Females_L</t>
+  </si>
+  <si>
+    <t>HM2_Males_L</t>
+  </si>
+  <si>
+    <t>HM1_C</t>
+  </si>
+  <si>
+    <t>HM2_Females_C</t>
+  </si>
+  <si>
+    <t>HM2_Males_C</t>
+  </si>
+  <si>
+    <t>DHE_MCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_MCS2_Males</t>
+  </si>
+  <si>
+    <t>DHE_PCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_PCS2_Males</t>
+  </si>
+  <si>
+    <t>DLS2_Females</t>
+  </si>
+  <si>
+    <t>DLS2_Males</t>
   </si>
 </sst>
 </file>
@@ -454,13 +487,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,7 +501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -476,7 +509,7 @@
         <v>0.81346415014080209</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -484,7 +517,7 @@
         <v>0.82562018838448625</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -492,7 +525,7 @@
         <v>0.53166683592248576</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -500,7 +533,7 @@
         <v>0.64173720769193388</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -508,7 +541,7 @@
         <v>1.7533164842397457</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -516,7 +549,7 @@
         <v>3.737785387161713</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -524,7 +557,7 @@
         <v>6.6133857070747402</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -532,7 +565,7 @@
         <v>1.1671</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -540,7 +573,7 @@
         <v>1.2093</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -548,7 +581,7 @@
         <v>0.98887999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -556,7 +589,7 @@
         <v>0.95128999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
@@ -564,7 +597,7 @@
         <v>1.2788999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
@@ -572,44 +605,129 @@
         <v>1.2788999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="1">
-        <v>4.4450300852579687</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="1">
-        <v>7.951543214267657</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>4.4468128085002929</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16">
+        <v>4.2769575506466175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B17">
-        <v>7.1364100298230317</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>3.7038567524111912</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18">
-        <v>1.2179012672192562</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B19" s="1">
         <v>1.528311</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20">
+        <v>2.5987714833007889</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21">
+        <v>2.1900536031824447</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>7.9559814188182223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23">
+        <v>7.2405551802300421</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24">
+        <v>6.4476832985046046</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25">
+        <v>7.1418652596474503</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26">
+        <v>6.1866366824002945</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27">
+        <v>5.5056435446648049</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28">
+        <v>2.0304724900805509</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>1.8025199770624896</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>1.6950010985371542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update regression estimates do-files and RMSE.xlsx
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCB00F9-F183-0147-BE8D-9FA44067C648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2804C8-D5BE-8D41-849C-2286B7E5F5D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="30240" windowHeight="19500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30280" yWindow="600" windowWidth="19640" windowHeight="19560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -64,13 +64,43 @@
     <t>HM1_L</t>
   </si>
   <si>
+    <t>HM2_Females_L</t>
+  </si>
+  <si>
+    <t>HM2_Males_L</t>
+  </si>
+  <si>
+    <t>HM2_Females_C</t>
+  </si>
+  <si>
+    <t>HM2_Males_C</t>
+  </si>
+  <si>
     <t>DHE_MCS1</t>
   </si>
   <si>
+    <t>DHE_MCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_MCS2_Males</t>
+  </si>
+  <si>
     <t>DHE_PCS1</t>
   </si>
   <si>
+    <t>DHE_PCS2_Females</t>
+  </si>
+  <si>
+    <t>DHE_PCS2_Males</t>
+  </si>
+  <si>
     <t>DLS1</t>
+  </si>
+  <si>
+    <t>DLS2_Females</t>
+  </si>
+  <si>
+    <t>DLS2_Males</t>
   </si>
   <si>
     <t>C1b</t>
@@ -448,8 +478,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="30.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -464,7 +497,7 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.81331302800611116</v>
+        <v>0.81965385041030181</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -472,7 +505,7 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.82615669757546539</v>
+        <v>0.82891267508318089</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -480,7 +513,7 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>0.53163272118969074</v>
+        <v>0.5280315538367093</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -488,7 +521,7 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>0.64176230754993757</v>
+        <v>0.6384628582929639</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -496,7 +529,7 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <v>1.7533164842397457</v>
+        <v>1.7483244903591919</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -504,7 +537,7 @@
         <v>3</v>
       </c>
       <c r="B7">
-        <v>3.737785387161713</v>
+        <v>3.7551118303514497</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -512,7 +545,7 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <v>6.5920042103174792</v>
+        <v>6.4899407537254499</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -520,7 +553,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>1.0359298734760334</v>
+        <v>1.0366118799278699</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -548,19 +581,19 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="1">
-        <v>4.4450300852579687</v>
+      <c r="B13">
+        <v>4.4456117642900459</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="1">
-        <v>7.951543214267657</v>
+      <c r="B14">
+        <v>4.2766564624169652</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -568,7 +601,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>7.1364100298230317</v>
+        <v>3.7039324632313728</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -576,14 +609,94 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>1.2179012672192562</v>
+        <v>2.5977267935063337</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17">
+        <v>2.1895888225015536</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>7.9661177286442255</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>7.1714148232921389</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>6.4840573935244814</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21">
+        <v>7.0657713186475233</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22">
+        <v>6.0610553268076588</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>5.4194767626250133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24">
+        <v>1.9023687544636687</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>1.7145370168869383</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>1.6259752837992298</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1">
         <v>1.528311</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct bugs in Excel files and update regressor names
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,19 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F31421A-A2A9-134E-BAE0-B0FAE2CD5120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="UK" sheetId="1" r:id="rId2"/>
+    <sheet name="UK" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -21,18 +28,6 @@
     <t>COEFFICIENT</t>
   </si>
   <si>
-    <t>Wages_FemalesNE</t>
-  </si>
-  <si>
-    <t>Wages_MalesNE</t>
-  </si>
-  <si>
-    <t>Wages_FemalesE</t>
-  </si>
-  <si>
-    <t>Wages_MalesE</t>
-  </si>
-  <si>
     <t>I1b</t>
   </si>
   <si>
@@ -106,16 +101,24 @@
   </si>
   <si>
     <t>DLS2_Males</t>
+  </si>
+  <si>
+    <t>C1b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -138,21 +141,347 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -160,206 +489,215 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>0.81857066434101511</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>0.83183050833110173</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>0.52838226151512502</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>0.63794775886311106</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B6">
         <v>1.7487317224564645</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>3.7549875108949018</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B8">
         <v>6.4764075049781749</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>1.0366118799278699</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>0.85170355381228569</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>1.1480377870969753</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>1.1960390964496237</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B13">
         <v>4.460523583140219</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>4.2529536919897684</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>3.7382957371324035</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>2.5977267935063337</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>2.1895888225015536</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>7.9661177286442255</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B19">
         <v>7.1714148232921389</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B20">
         <v>6.4840573935244814</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B21">
         <v>7.0657713186475233</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B22">
         <v>6.0610553268076588</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B23">
         <v>5.4194767626250133</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B24">
         <v>1.9023687544636687</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B25">
         <v>1.7145370168869383</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B26">
         <v>1.6259752837992298</v>
       </c>
     </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1.528311</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add estimates with time dummies
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F31421A-A2A9-134E-BAE0-B0FAE2CD5120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B953F3-C7FF-784E-A160-3C0AC51F71C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34980" yWindow="600" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -526,7 +526,7 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <v>1.7487317224564645</v>
+        <v>1.742377978839817</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -534,7 +534,7 @@
         <v>3</v>
       </c>
       <c r="B7">
-        <v>3.7549875108949018</v>
+        <v>3.7543598400770608</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -542,7 +542,7 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <v>6.4764075049781749</v>
+        <v>6.4557322480400128</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Remove C1b value from RMSE
Stop applying regression RMSE and random Gaussian draws to the childcare cost (C1b) regression. In the latest estimate update, C1b was no longer included in RMSE. The old value lingered for the sake of code functioning. With this commit, the code is updated accordingly.
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F31421A-A2A9-134E-BAE0-B0FAE2CD5120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08ABB30-1DD5-C84C-AD17-7F8C5D8A1E3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>DLS2_Males</t>
-  </si>
-  <si>
-    <t>C1b</t>
   </si>
 </sst>
 </file>
@@ -478,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -562,7 +559,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B11">
@@ -687,14 +684,6 @@
       </c>
       <c r="B26">
         <v>1.6259752837992298</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" s="1">
-        <v>1.528311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>